<commit_message>
docs: add sprint 2 backlog detailed technical breakdown and sync excel
</commit_message>
<xml_diff>
--- a/docs/Product_Backlog_HRM_ictu.xlsx
+++ b/docs/Product_Backlog_HRM_ictu.xlsx
@@ -4,11 +4,12 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlogs" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 2" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1844,7 +1845,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -1870,7 +1871,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -1896,7 +1897,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -1922,7 +1923,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -1952,7 +1953,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1979,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2004,7 +2005,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2030,7 +2031,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2056,7 +2057,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2082,7 +2083,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2109,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2139,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2165,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2190,7 +2191,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2217,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2243,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2268,7 +2269,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2298,7 +2299,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2324,7 +2325,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2350,7 +2351,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2376,7 +2377,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2402,7 +2403,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2432,7 +2433,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2458,7 +2459,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2484,7 +2485,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2514,7 +2515,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2540,7 +2541,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2566,7 +2567,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2596,7 +2597,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2622,7 +2623,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đã xong</t>
         </is>
       </c>
     </row>
@@ -2639,4 +2640,888 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="39.43" customWidth="1" min="1" max="1"/>
+    <col width="85" customWidth="1" min="2" max="2"/>
+    <col width="22.43" customWidth="1" min="3" max="3"/>
+    <col width="23.29" customWidth="1" min="4" max="4"/>
+    <col width="26.29" customWidth="1" min="5" max="5"/>
+    <col width="27.86" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Task (Phân rã User Story thành các nhiệm vụ nhỏ)</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Priority 
+ (Cao/Trung/Thấp)</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Estimate 
+ (Story Point/giờ)</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Assign</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>Status 
+ (To Do / In Progress / Done)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>US 7.0: Chỉnh sửa thông tin phòng ban</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>BE: Xây dựng API PUT /api/departments/:id cập nhật thông tin phòng ban, validate trùng mã</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Hà Sỹ Nguyên (BE)</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="10" t="n"/>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>FE: Nâng cấp modal Form Chỉnh sửa phòng ban, prefill dữ liệu cũ &amp; gọi API PUT</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Nguyễn Minh Lượng (FE)</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="11" t="n"/>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>QA: Viết Test Cases &amp; kiểm thử luồng Chỉnh sửa phòng ban (đổi tên, đổi SĐT, kiểm tra ràng buộc)</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Hoàng Văn Khuyến (QA)</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>US 13.0: Cập nhật thông tin nhân sự</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>BE: Xây dựng API PUT /api/employees/:id cập nhật chức vụ, mức lương, số điện thoại</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Đào Đức Mạnh (BE)</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="10" t="n"/>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>FE: Dựng Modal chỉnh sửa hồ sơ nhân viên, hỗ trợ chọn phòng ban từ dropdown &amp; gọi API</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Hoàng Minh Khánh (FE)</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>QA: Kiểm thử cập nhật thông tin nhân viên, xác nhận không làm ảnh hưởng đến trường CCCD mã hóa</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Hoàng Văn Khuyến (QA)</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>US 14.0: Thôi việc nhân viên (Soft-delete)</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>BE: Xây dựng API DELETE/PATCH /api/employees/:id đổi trạng thái Resigned &amp; khóa tài khoản user</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Đoàn Ngọc Mạnh (BE)</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="10" t="n"/>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>FE: Dựng nút hành động Thôi việc trên bảng nhân sự, popup cảnh báo xác nhận trước khi cập nhật</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Nguyễn Minh Lượng (FE)</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>QA: Kiểm thử luồng Thôi việc, xác nhận nhân viên không bị xóa vĩnh viễn khỏi CSDL và không thể login</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Triệu Quốc Khánh (QA)</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>US 19.0: Lịch sử chấm công theo tháng</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>BE: Xây dựng API GET /api/attendance/history lọc theo tháng/năm, tính tổng ngày công, đi muộn, về sớm</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Hà Sỹ Nguyên (BE)</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="10" t="n"/>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>FE: Dựng giao diện Bảng lịch sử chấm công theo tháng (bộ chọn tháng/năm, bảng chi tiết từng ngày)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Vũ Thị Thanh Ngân (FE)</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>QA: Kiểm thử độ chính xác của thuật toán tính tổng ngày công và đối soát dữ liệu lịch sử</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Ngô Đức Khải (QA)</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>US 20.0: Dashboard tổng quan nhân sự</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>BE: Xây dựng API GET /api/dashboard/stats tổng hợp KPI tổng nhân sự, số PB, tỷ lệ có mặt hôm nay</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Đoàn Ngọc Mạnh (BE)</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="10" t="n"/>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>FE: Dựng 3 thẻ thống kê KPI thực tế trên Dashboard &amp; biểu đồ phân bổ nhân sự từng phòng ban</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Nguyễn Minh Lượng (FE)</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>QA: Kiểm thử số liệu thống kê trên Dashboard đối chiếu chính xác 100% với dữ liệu database</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>Triệu Quốc Khánh (QA)</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>US 22.0: Xuất báo cáo chấm công</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>BE: Xây dựng API GET /api/reports/attendance/export xuất bảng tổng hợp công ra file Excel/CSV</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Đào Đức Mạnh (BE)</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="10" t="n"/>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>FE: Tích hợp nút 'Xuất báo cáo Excel' trên giao diện chấm công, xử lý tải file mượt mà</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Vũ Thị Thanh Ngân (FE)</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="11" t="n"/>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>QA: Kiểm thử tải file báo cáo, mở file đối soát font tiếng Việt UTF-8 và số liệu công</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Ngô Đức Khải (QA)</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>US 3.0: Đổi mật khẩu cá nhân</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>BE: Xây dựng API PUT /api/auth/change-password xác thực mật khẩu cũ và băm bcrypt mật khẩu mới</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Đào Đức Mạnh (BE)</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="10" t="n"/>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>FE: Dựng Modal Đổi mật khẩu cá nhân, validate mật khẩu mới trùng khớp và độ phức tạp</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>Hoàng Minh Khánh (FE)</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="11" t="n"/>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>QA: Kiểm thử các ca biên đổi mật khẩu (sai mật khẩu cũ, mật khẩu mới quá ngắn, đăng nhập lại)</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>Hoàng Văn Khuyến (QA)</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>US 29.0: Giám sát Prometheus + Grafana (Commit 2)</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>DevOps: Thiết lập kiến trúc mạng đa tầng tách biệt: app-network và monitoring trong docker-compose</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Đỗ Quang Minh (SM)</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="10" t="n"/>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>DevOps: Triển khai container mysqld-exporter:v0.14.0 (port 9104) kết nối MySQL lấy số liệu CSDL</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Đỗ Quang Minh (SM)</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="10" t="n"/>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>DevOps: Triển khai container cadvisor (port 8080) và node-exporter (port 9100) thu thập metrics hệ thống</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>Đỗ Quang Minh (SM)</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="10" t="n"/>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>DevOps: Cấu hình prometheus.yml scrape 5 targets (Prometheus, Node, cAdvisor, MySQL Exporter, App)</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Đỗ Quang Minh (SM)</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="10" t="n"/>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>SRE: Triển khai container grafana:latest (port 3000) với Datasource Provisioning tự động nạp Prometheus</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>Đỗ Quang Minh (SM)</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="10" t="n"/>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>SRE: Import &amp; cấu hình 3 Dashboards Grafana: Node Exporter (1860), Docker (14282), MySQL Overview (7362)</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>Đỗ Quang Minh (SM)</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="11" t="n"/>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>QA: Kiểm tra xác nhận 5/5 targets Prometheus đều UP và số liệu hiển thị realtime trên Grafana</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>Triệu Quốc Khánh (QA)</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Nghiệm thu Sprint 2 &amp; Commit 2</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>QA: Kiểm thử tích hợp E2E toàn bộ chức năng Sprint 2 trên môi trường Docker Compose</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>Hoàng Văn Khuyến (QA)</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="11" t="n"/>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>SM: Rà soát Sprint Goal 2, cập nhật tài liệu kỹ thuật và thực hiện Commit 2 lên GitHub</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Cao</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>Đỗ Quang Minh (SM)</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="A20:A22"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="A23:A29"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="A30:A31"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>